<commit_message>
chore: align with Lake Protocol v8.1.5
</commit_message>
<xml_diff>
--- a/docs/vaults/u1-aa-01-applied-econometrics/ape2-crisis-iess/analysis_erick_condoy/reports/unit_root_tests.xlsx
+++ b/docs/vaults/u1-aa-01-applied-econometrics/ape2-crisis-iess/analysis_erick_condoy/reports/unit_root_tests.xlsx
@@ -14,123 +14,126 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
-  <si>
-    <t>(ADF)</t>
-  </si>
-  <si>
-    <t>(PP)</t>
-  </si>
-  <si>
-    <t>(ZA)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="41">
+  <si>
+    <t>Serie</t>
+  </si>
+  <si>
+    <t>ADF</t>
+  </si>
+  <si>
+    <t>PP</t>
+  </si>
+  <si>
+    <t>ZA</t>
   </si>
   <si>
     <t>Break</t>
   </si>
   <si>
+    <t>I(d)</t>
+  </si>
+  <si>
     <t>AF</t>
   </si>
   <si>
+    <t>GM</t>
+  </si>
+  <si>
+    <t>MI</t>
+  </si>
+  <si>
+    <t>HO</t>
+  </si>
+  <si>
     <t>FL</t>
   </si>
   <si>
-    <t>EM</t>
-  </si>
-  <si>
-    <t>GDP</t>
-  </si>
-  <si>
-    <t>SBU</t>
-  </si>
-  <si>
-    <t>-1.196</t>
-  </si>
-  <si>
-    <t>-2.269</t>
-  </si>
-  <si>
-    <t>-2.470</t>
-  </si>
-  <si>
-    <t>-1.604*</t>
-  </si>
-  <si>
-    <t>-0.961</t>
-  </si>
-  <si>
-    <t>-0.568</t>
-  </si>
-  <si>
-    <t>-2.637</t>
-  </si>
-  <si>
-    <t>-4.815</t>
-  </si>
-  <si>
-    <t>-1.599***</t>
-  </si>
-  <si>
-    <t>-4.038***</t>
-  </si>
-  <si>
-    <t>-5.159**</t>
-  </si>
-  <si>
-    <t>-3.414</t>
-  </si>
-  <si>
-    <t>-5.363**</t>
-  </si>
-  <si>
-    <t>-3.660</t>
-  </si>
-  <si>
-    <t>-15.022***</t>
-  </si>
-  <si>
-    <t>-1.460</t>
-  </si>
-  <si>
-    <t>-3.169</t>
-  </si>
-  <si>
-    <t>-3.819</t>
-  </si>
-  <si>
-    <t>-3.390*</t>
-  </si>
-  <si>
-    <t>-2.522</t>
-  </si>
-  <si>
-    <t>-1.755</t>
-  </si>
-  <si>
-    <t>-5.451</t>
-  </si>
-  <si>
-    <t>-7.445</t>
-  </si>
-  <si>
-    <t>-4.544***</t>
-  </si>
-  <si>
-    <t>-7.455***</t>
-  </si>
-  <si>
-    <t>-4.771</t>
-  </si>
-  <si>
-    <t>-5.901***</t>
-  </si>
-  <si>
-    <t>-5.225**</t>
-  </si>
-  <si>
-    <t>-4.490</t>
-  </si>
-  <si>
-    <t>-11.610***</t>
+    <t>-1.529</t>
+  </si>
+  <si>
+    <t>-0.863</t>
+  </si>
+  <si>
+    <t>-3.269</t>
+  </si>
+  <si>
+    <t>-2.264</t>
+  </si>
+  <si>
+    <t>-2.423</t>
+  </si>
+  <si>
+    <t>-1.367</t>
+  </si>
+  <si>
+    <t>-1.566</t>
+  </si>
+  <si>
+    <t>-2.220</t>
+  </si>
+  <si>
+    <t>-1.154</t>
+  </si>
+  <si>
+    <t>-2.785</t>
+  </si>
+  <si>
+    <t>-2.707</t>
+  </si>
+  <si>
+    <t>-4.458</t>
+  </si>
+  <si>
+    <t>-5.665***</t>
+  </si>
+  <si>
+    <t>-3.791</t>
+  </si>
+  <si>
+    <t>-3.657</t>
+  </si>
+  <si>
+    <t>-1.936</t>
+  </si>
+  <si>
+    <t>-3.817*</t>
+  </si>
+  <si>
+    <t>-4.347**</t>
+  </si>
+  <si>
+    <t>-4.212**</t>
+  </si>
+  <si>
+    <t>-2.963</t>
+  </si>
+  <si>
+    <t>-8.747***</t>
+  </si>
+  <si>
+    <t>-3.544*</t>
+  </si>
+  <si>
+    <t>-3.128</t>
+  </si>
+  <si>
+    <t>-6.756***</t>
+  </si>
+  <si>
+    <t>-4.578</t>
+  </si>
+  <si>
+    <t>-10.371***</t>
+  </si>
+  <si>
+    <t>-9.270***</t>
+  </si>
+  <si>
+    <t>-4.308</t>
+  </si>
+  <si>
+    <t>-7.020***</t>
   </si>
   <si>
     <t>I(1)</t>
@@ -469,189 +472,195 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" t="s">
-        <v>2</v>
-      </c>
       <c r="I1" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="J1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E2">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I2">
-        <v>2013</v>
+        <v>2008</v>
       </c>
       <c r="J2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3">
-        <v>2015</v>
+        <v>2008</v>
       </c>
       <c r="F3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I3">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="J3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E4">
+        <v>2016</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4">
         <v>2019</v>
       </c>
-      <c r="F4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4">
-        <v>2010</v>
-      </c>
       <c r="J4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E5">
-        <v>2013</v>
+        <v>1998</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I5">
         <v>2011</v>
       </c>
       <c r="J5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>2014</v>
+        <v>2009</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I6">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="J6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>